<commit_message>
feat: realistic submission content across all 25 parsing fixtures
</commit_message>
<xml_diff>
--- a/samples/fixtures/xlsx/losses-table.xlsx
+++ b/samples/fixtures/xlsx/losses-table.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,6 +432,11 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Cause</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -447,6 +452,11 @@
           <t>settled</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>water damage, Hull depot</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -460,6 +470,71 @@
       <c r="C3" t="inlineStr">
         <is>
           <t>settled</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>forklift impact, Quay Street</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2021-09-14</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>storm ingress, Dockside</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2020-01-22</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>handling damage, Port Road</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2019-05-30</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>900</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>pilferage, Beta Dock</t>
         </is>
       </c>
     </row>

</xml_diff>